<commit_message>
feat: complete R01-R69 acceptance evidence pack
</commit_message>
<xml_diff>
--- a/files/R01-R69全节点业务验收测试包/00_使用说明与总目录/M00_M00-DIR-001_TEST-M00-004_资料总目录.xlsx
+++ b/files/R01-R69全节点业务验收测试包/00_使用说明与总目录/M00_M00-DIR-001_TEST-M00-004_资料总目录.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料总目录" sheetId="1" r:id="R10dc8bac141b4729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖统计" sheetId="2" r:id="R79e072afebc044f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料总目录" sheetId="1" r:id="R030f23d9fd1e42fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖统计" sheetId="2" r:id="Rfed913361d8148ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +43,7 @@
       <x:name val="Arial Unicode MS"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -60,8 +60,13 @@
         <x:fgColor rgb="FFFCE8E6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:left/>
@@ -91,11 +96,63 @@
       <x:right/>
       <x:bottom/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFE6A7A2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="69">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -187,6 +244,70 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -238,6 +359,70 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2190750" cy="876300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="a7a86fef-6e02-4035-a1ff-39c842c5b6f0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb35711206f5140f8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2190750" cy="876300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="5417cbec-3d69-4fc1-ae31-19d4761fd689"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf69e0813e5540d1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -437,7 +622,7 @@
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20.329999923706055" hidden="0" customWidth="1"/>
@@ -566,33 +751,33 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="35" t="str">
-        <x:v>B00-DESIGN-001</x:v>
+        <x:v>M00-SOURCE-001</x:v>
       </x:c>
       <x:c r="B9" s="36" t="str">
-        <x:v>B00</x:v>
+        <x:v>M00</x:v>
       </x:c>
       <x:c r="C9" s="36" t="str">
-        <x:v>基础设计输入摘要</x:v>
+        <x:v>原始证据来源与页级绑定台账</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E9" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F9" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-B00-001</x:v>
+        <x:v>TEST-M00-005</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="35" t="str">
-        <x:v>B00-CONSTRUCTION-001</x:v>
+        <x:v>M00-DATA-001</x:v>
       </x:c>
       <x:c r="B10" s="36" t="str">
-        <x:v>B00</x:v>
+        <x:v>M00</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:v>施工组织设计</x:v>
+        <x:v>数据一致性差异与闭环报告</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -601,98 +786,98 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F10" s="37" t="str">
-        <x:v>TEST-B00-002</x:v>
+        <x:v>TEST-M00-006</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="35" t="str">
-        <x:v>B00-QUALITY-001</x:v>
+        <x:v>M00-SEAL-001</x:v>
       </x:c>
       <x:c r="B11" s="36" t="str">
-        <x:v>B00</x:v>
+        <x:v>M00</x:v>
       </x:c>
       <x:c r="C11" s="36" t="str">
-        <x:v>质量计划</x:v>
+        <x:v>测试专用签章样式与使用登记台账</x:v>
       </x:c>
       <x:c r="D11" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E11" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F11" s="37" t="str">
-        <x:v>TEST-B00-003</x:v>
+        <x:v>TEST-M00-007</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="35" t="str">
-        <x:v>B00-QUAL-001</x:v>
+        <x:v>B00-DESIGN-001</x:v>
       </x:c>
       <x:c r="B12" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C12" s="36" t="str">
-        <x:v>单位人员资质台账</x:v>
+        <x:v>基础设计输入摘要</x:v>
       </x:c>
       <x:c r="D12" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E12" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F12" s="37" t="str">
-        <x:v>TEST-B00-004</x:v>
+        <x:v>QX201903S-13-Y-TEST-B00-001</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="35" t="str">
-        <x:v>B00-LINES-001</x:v>
+        <x:v>B00-CONSTRUCTION-001</x:v>
       </x:c>
       <x:c r="B13" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C13" s="36" t="str">
-        <x:v>基础管线台账</x:v>
+        <x:v>施工组织设计</x:v>
       </x:c>
       <x:c r="D13" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E13" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F13" s="37" t="str">
-        <x:v>TEST-B00-005</x:v>
+        <x:v>TEST-B00-002</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="35" t="str">
-        <x:v>B00-MATERIAL-001</x:v>
+        <x:v>B00-QUALITY-001</x:v>
       </x:c>
       <x:c r="B14" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C14" s="36" t="str">
-        <x:v>材料验收台账</x:v>
+        <x:v>质量计划</x:v>
       </x:c>
       <x:c r="D14" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E14" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F14" s="37" t="str">
-        <x:v>TEST-B00-006</x:v>
+        <x:v>TEST-B00-003</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="35" t="str">
-        <x:v>B00-VALVE-001</x:v>
+        <x:v>B00-QUAL-001</x:v>
       </x:c>
       <x:c r="B15" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C15" s="36" t="str">
-        <x:v>阀门耐压试验记录</x:v>
+        <x:v>单位人员资质台账</x:v>
       </x:c>
       <x:c r="D15" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -701,38 +886,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F15" s="37" t="str">
-        <x:v>TEST-B00-007</x:v>
+        <x:v>TEST-B00-004</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="35" t="str">
-        <x:v>B00-WELD-001</x:v>
+        <x:v>B00-LINES-001</x:v>
       </x:c>
       <x:c r="B16" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C16" s="36" t="str">
-        <x:v>PQR-WPS基础包</x:v>
+        <x:v>基础管线台账</x:v>
       </x:c>
       <x:c r="D16" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E16" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F16" s="37" t="str">
-        <x:v>TEST-B00-008</x:v>
+        <x:v>TEST-B00-005</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="35" t="str">
-        <x:v>B00-WELD-LEDGER-001</x:v>
+        <x:v>B00-MATERIAL-001</x:v>
       </x:c>
       <x:c r="B17" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C17" s="36" t="str">
-        <x:v>焊口与检验台账</x:v>
+        <x:v>材料验收台账</x:v>
       </x:c>
       <x:c r="D17" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -741,38 +926,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F17" s="37" t="str">
-        <x:v>TEST-B00-009</x:v>
+        <x:v>TEST-B00-006</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="35" t="str">
-        <x:v>B00-NDT-001</x:v>
+        <x:v>B00-VALVE-001</x:v>
       </x:c>
       <x:c r="B18" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C18" s="36" t="str">
-        <x:v>基础无损检测报告</x:v>
+        <x:v>阀门耐压试验记录</x:v>
       </x:c>
       <x:c r="D18" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E18" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F18" s="37" t="str">
-        <x:v>TEST-B00-010</x:v>
+        <x:v>TEST-B00-007</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="35" t="str">
-        <x:v>B00-TEST-001</x:v>
+        <x:v>B00-WELD-001</x:v>
       </x:c>
       <x:c r="B19" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C19" s="36" t="str">
-        <x:v>压力与泄漏试验方案</x:v>
+        <x:v>PQR-WPS基础包</x:v>
       </x:c>
       <x:c r="D19" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -781,18 +966,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F19" s="37" t="str">
-        <x:v>TEST-B00-011</x:v>
+        <x:v>TEST-B00-008</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="35" t="str">
-        <x:v>B00-INSTALL-001</x:v>
+        <x:v>B00-WELD-LEDGER-001</x:v>
       </x:c>
       <x:c r="B20" s="36" t="str">
         <x:v>B00</x:v>
       </x:c>
       <x:c r="C20" s="36" t="str">
-        <x:v>安装试验吹扫综合记录</x:v>
+        <x:v>焊口与检验台账</x:v>
       </x:c>
       <x:c r="D20" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -801,18 +986,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F20" s="37" t="str">
-        <x:v>TEST-B00-012</x:v>
+        <x:v>TEST-B00-009</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="35" t="str">
-        <x:v>S01-DESIGN-001</x:v>
+        <x:v>B00-NDT-001</x:v>
       </x:c>
       <x:c r="B21" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C21" s="36" t="str">
-        <x:v>境外与新材料设计变更</x:v>
+        <x:v>基础无损检测报告</x:v>
       </x:c>
       <x:c r="D21" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -821,18 +1006,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F21" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S01-001</x:v>
+        <x:v>TEST-B00-010</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="35" t="str">
-        <x:v>S01-FOREIGN-001</x:v>
+        <x:v>B00-TEST-001</x:v>
       </x:c>
       <x:c r="B22" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C22" s="36" t="str">
-        <x:v>境外制造与型式资料</x:v>
+        <x:v>压力与泄漏试验方案</x:v>
       </x:c>
       <x:c r="D22" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -841,178 +1026,178 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F22" s="37" t="str">
-        <x:v>TEST-S01-002</x:v>
+        <x:v>TEST-B00-011</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="35" t="str">
-        <x:v>S01-MATERIAL-001</x:v>
+        <x:v>B00-INSTALL-001</x:v>
       </x:c>
       <x:c r="B23" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C23" s="36" t="str">
-        <x:v>企业标准与材料证明</x:v>
+        <x:v>安装试验吹扫综合记录</x:v>
       </x:c>
       <x:c r="D23" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E23" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F23" s="37" t="str">
-        <x:v>TEST-S01-003</x:v>
+        <x:v>TEST-B00-012</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="35" t="str">
-        <x:v>S01-RETEST-001</x:v>
+        <x:v>B00-PHOTO-001</x:v>
       </x:c>
       <x:c r="B24" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C24" s="36" t="str">
-        <x:v>验证性复验记录</x:v>
+        <x:v>管道组对现场核验图</x:v>
       </x:c>
       <x:c r="D24" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E24" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F24" s="37" t="str">
-        <x:v>TEST-S01-004</x:v>
+        <x:v>TEST-B00-013</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="35" t="str">
-        <x:v>S01-REVIEW-001</x:v>
+        <x:v>B00-PHOTO-002</x:v>
       </x:c>
       <x:c r="B25" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C25" s="36" t="str">
-        <x:v>新材料评审批准</x:v>
+        <x:v>焊缝外观现场核验图</x:v>
       </x:c>
       <x:c r="D25" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E25" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F25" s="37" t="str">
-        <x:v>TEST-S01-005</x:v>
+        <x:v>TEST-B00-014</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="35" t="str">
-        <x:v>S01-ACCEPT-001</x:v>
+        <x:v>B00-PHOTO-003</x:v>
       </x:c>
       <x:c r="B26" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C26" s="36" t="str">
-        <x:v>到货验收记录</x:v>
+        <x:v>无损检测现场核验图</x:v>
       </x:c>
       <x:c r="D26" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E26" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F26" s="37" t="str">
-        <x:v>TEST-S01-006</x:v>
+        <x:v>TEST-B00-015</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="35" t="str">
-        <x:v>S01-MARK-001</x:v>
+        <x:v>B00-PHOTO-004</x:v>
       </x:c>
       <x:c r="B27" s="36" t="str">
-        <x:v>S01</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C27" s="36" t="str">
-        <x:v>标志移植台账</x:v>
+        <x:v>防腐补伤现场核验图</x:v>
       </x:c>
       <x:c r="D27" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E27" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F27" s="37" t="str">
-        <x:v>TEST-S01-007</x:v>
+        <x:v>TEST-B00-016</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="35" t="str">
-        <x:v>S02-DESIGN-001</x:v>
+        <x:v>B00-FILM-001</x:v>
       </x:c>
       <x:c r="B28" s="36" t="str">
-        <x:v>S02</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C28" s="36" t="str">
-        <x:v>材料代用设计变更</x:v>
+        <x:v>PL8303射线检测模拟底片</x:v>
       </x:c>
       <x:c r="D28" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E28" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F28" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S02-001</x:v>
+        <x:v>TEST-B00-017</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="35" t="str">
-        <x:v>S02-CALC-001</x:v>
+        <x:v>B00-FILM-002</x:v>
       </x:c>
       <x:c r="B29" s="36" t="str">
-        <x:v>S02</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C29" s="36" t="str">
-        <x:v>技术比较与强度校核</x:v>
+        <x:v>PL8306射线检测模拟底片</x:v>
       </x:c>
       <x:c r="D29" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E29" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F29" s="37" t="str">
-        <x:v>TEST-S02-002</x:v>
+        <x:v>TEST-B00-018</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="35" t="str">
-        <x:v>S02-APPROVAL-001</x:v>
+        <x:v>B00-QUERY-001</x:v>
       </x:c>
       <x:c r="B30" s="36" t="str">
-        <x:v>S02</x:v>
+        <x:v>B00</x:v>
       </x:c>
       <x:c r="C30" s="36" t="str">
-        <x:v>材料代用书面批准</x:v>
+        <x:v>焊工资格外部查询测试截图</x:v>
       </x:c>
       <x:c r="D30" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E30" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
-        <x:v>TEST-S02-003</x:v>
+        <x:v>TEST-B00-019</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="35" t="str">
-        <x:v>S02-WPS-001</x:v>
+        <x:v>S01-DESIGN-001</x:v>
       </x:c>
       <x:c r="B31" s="36" t="str">
-        <x:v>S02</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C31" s="36" t="str">
-        <x:v>替代材料与WPS适用性</x:v>
+        <x:v>境外与新材料设计变更</x:v>
       </x:c>
       <x:c r="D31" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1021,38 +1206,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F31" s="37" t="str">
-        <x:v>TEST-S02-004</x:v>
+        <x:v>QX201903S-13-Y-TEST-S01-001</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="35" t="str">
-        <x:v>S02-INSTALL-001</x:v>
+        <x:v>S01-FOREIGN-001</x:v>
       </x:c>
       <x:c r="B32" s="36" t="str">
-        <x:v>S02</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C32" s="36" t="str">
-        <x:v>替代材料验收安装记录</x:v>
+        <x:v>境外制造与型式资料</x:v>
       </x:c>
       <x:c r="D32" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E32" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F32" s="37" t="str">
-        <x:v>TEST-S02-005</x:v>
+        <x:v>TEST-S01-002</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="35" t="str">
-        <x:v>S03-DESIGN-001</x:v>
+        <x:v>S01-MATERIAL-001</x:v>
       </x:c>
       <x:c r="B33" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C33" s="36" t="str">
-        <x:v>热处理管线设计变更与计算</x:v>
+        <x:v>企业标准与材料证明</x:v>
       </x:c>
       <x:c r="D33" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1061,58 +1246,58 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F33" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S03-001</x:v>
+        <x:v>TEST-S01-003</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="35" t="str">
-        <x:v>S03-WPS-001</x:v>
+        <x:v>S01-RETEST-001</x:v>
       </x:c>
       <x:c r="B34" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C34" s="36" t="str">
-        <x:v>PQR-WPS专项包</x:v>
+        <x:v>验证性复验记录</x:v>
       </x:c>
       <x:c r="D34" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E34" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F34" s="37" t="str">
-        <x:v>TEST-S03-002</x:v>
+        <x:v>TEST-S01-004</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="35" t="str">
-        <x:v>S03-WELDER-001</x:v>
+        <x:v>S01-REVIEW-001</x:v>
       </x:c>
       <x:c r="B35" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C35" s="36" t="str">
-        <x:v>焊工焊材台账</x:v>
+        <x:v>新材料评审批准</x:v>
       </x:c>
       <x:c r="D35" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E35" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F35" s="37" t="str">
-        <x:v>TEST-S03-003</x:v>
+        <x:v>TEST-S01-005</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="35" t="str">
-        <x:v>S03-WELDLOG-001</x:v>
+        <x:v>S01-ACCEPT-001</x:v>
       </x:c>
       <x:c r="B36" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C36" s="36" t="str">
-        <x:v>焊口施焊台账</x:v>
+        <x:v>到货验收记录</x:v>
       </x:c>
       <x:c r="D36" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -1121,58 +1306,58 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F36" s="37" t="str">
-        <x:v>TEST-S03-004</x:v>
+        <x:v>TEST-S01-006</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="35" t="str">
-        <x:v>S03-NDT-INITIAL-001</x:v>
+        <x:v>S01-MARK-001</x:v>
       </x:c>
       <x:c r="B37" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C37" s="36" t="str">
-        <x:v>首次无损检测不合格报告</x:v>
+        <x:v>标志移植台账</x:v>
       </x:c>
       <x:c r="D37" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E37" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F37" s="37" t="str">
-        <x:v>TEST-S03-005</x:v>
+        <x:v>TEST-S01-007</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="35" t="str">
-        <x:v>S03-REPAIR-001</x:v>
+        <x:v>S01-PHOTO-001</x:v>
       </x:c>
       <x:c r="B38" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S01</x:v>
       </x:c>
       <x:c r="C38" s="36" t="str">
-        <x:v>返修方案与记录</x:v>
+        <x:v>到货与标志移植核验图</x:v>
       </x:c>
       <x:c r="D38" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E38" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F38" s="37" t="str">
-        <x:v>TEST-S03-006</x:v>
+        <x:v>TEST-S01-008</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="35" t="str">
-        <x:v>S03-NDT-REPEAT-001</x:v>
+        <x:v>S02-DESIGN-001</x:v>
       </x:c>
       <x:c r="B39" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S02</x:v>
       </x:c>
       <x:c r="C39" s="36" t="str">
-        <x:v>返修复检合格报告</x:v>
+        <x:v>材料代用设计变更</x:v>
       </x:c>
       <x:c r="D39" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1181,18 +1366,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F39" s="37" t="str">
-        <x:v>TEST-S03-007</x:v>
+        <x:v>QX201903S-13-Y-TEST-S02-001</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="35" t="str">
-        <x:v>S03-PWHT-001</x:v>
+        <x:v>S02-CALC-001</x:v>
       </x:c>
       <x:c r="B40" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S02</x:v>
       </x:c>
       <x:c r="C40" s="36" t="str">
-        <x:v>热处理工艺与仪表</x:v>
+        <x:v>技术比较与强度校核</x:v>
       </x:c>
       <x:c r="D40" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1201,38 +1386,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F40" s="37" t="str">
-        <x:v>TEST-S03-008</x:v>
+        <x:v>TEST-S02-002</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="35" t="str">
-        <x:v>S03-PWHT-RECORD-001</x:v>
+        <x:v>S02-APPROVAL-001</x:v>
       </x:c>
       <x:c r="B41" s="36" t="str">
-        <x:v>S03</x:v>
+        <x:v>S02</x:v>
       </x:c>
       <x:c r="C41" s="36" t="str">
-        <x:v>热处理曲线与硬度记录</x:v>
+        <x:v>材料代用书面批准</x:v>
       </x:c>
       <x:c r="D41" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E41" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F41" s="37" t="str">
-        <x:v>TEST-S03-009</x:v>
+        <x:v>TEST-S02-003</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="35" t="str">
-        <x:v>S04-DESIGN-001</x:v>
+        <x:v>S02-WPS-001</x:v>
       </x:c>
       <x:c r="B42" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S02</x:v>
       </x:c>
       <x:c r="C42" s="36" t="str">
-        <x:v>穿越与阴极保护设计变更</x:v>
+        <x:v>替代材料与WPS适用性</x:v>
       </x:c>
       <x:c r="D42" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1241,78 +1426,78 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F42" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S04-001</x:v>
+        <x:v>TEST-S02-004</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="35" t="str">
-        <x:v>S04-DIAGRAM-001</x:v>
+        <x:v>S02-INSTALL-001</x:v>
       </x:c>
       <x:c r="B43" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S02</x:v>
       </x:c>
       <x:c r="C43" s="36" t="str">
-        <x:v>穿越结构与焊缝布置图</x:v>
+        <x:v>替代材料验收安装记录</x:v>
       </x:c>
       <x:c r="D43" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E43" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F43" s="37" t="str">
-        <x:v>TEST-S04-002</x:v>
+        <x:v>TEST-S02-005</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="35" t="str">
-        <x:v>S04-EQUIP-001</x:v>
+        <x:v>S03-DESIGN-001</x:v>
       </x:c>
       <x:c r="B44" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C44" s="36" t="str">
-        <x:v>设备材料台账</x:v>
+        <x:v>热处理管线设计变更与计算</x:v>
       </x:c>
       <x:c r="D44" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E44" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F44" s="37" t="str">
-        <x:v>TEST-S04-003</x:v>
+        <x:v>QX201903S-13-Y-TEST-S03-001</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="35" t="str">
-        <x:v>S04-INSTALL-001</x:v>
+        <x:v>S03-WPS-001</x:v>
       </x:c>
       <x:c r="B45" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C45" s="36" t="str">
-        <x:v>穿越施工与安装记录</x:v>
+        <x:v>PQR-WPS专项包</x:v>
       </x:c>
       <x:c r="D45" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E45" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F45" s="37" t="str">
-        <x:v>TEST-S04-004</x:v>
+        <x:v>TEST-S03-002</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="35" t="str">
-        <x:v>S04-CP-001</x:v>
+        <x:v>S03-WELDER-001</x:v>
       </x:c>
       <x:c r="B46" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C46" s="36" t="str">
-        <x:v>防腐阴保调试记录</x:v>
+        <x:v>焊工焊材台账</x:v>
       </x:c>
       <x:c r="D46" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -1321,38 +1506,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F46" s="37" t="str">
-        <x:v>TEST-S04-005</x:v>
+        <x:v>TEST-S03-003</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="35" t="str">
-        <x:v>S04-PHOTO-001</x:v>
+        <x:v>S03-WELDLOG-001</x:v>
       </x:c>
       <x:c r="B47" s="36" t="str">
-        <x:v>S04</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C47" s="36" t="str">
-        <x:v>施工照片</x:v>
+        <x:v>焊口施焊台账</x:v>
       </x:c>
       <x:c r="D47" s="36" t="str">
-        <x:v>JPG</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E47" s="36" t="str">
-        <x:v>JPG</x:v>
+        <x:v>PDF</x:v>
       </x:c>
       <x:c r="F47" s="37" t="str">
-        <x:v>TEST-S04-006</x:v>
+        <x:v>TEST-S03-004</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="35" t="str">
-        <x:v>S05-DESIGN-001</x:v>
+        <x:v>S03-NDT-INITIAL-001</x:v>
       </x:c>
       <x:c r="B48" s="36" t="str">
-        <x:v>S05</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C48" s="36" t="str">
-        <x:v>安全附件设计变更与选型</x:v>
+        <x:v>首次无损检测不合格报告</x:v>
       </x:c>
       <x:c r="D48" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1361,18 +1546,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F48" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S05-001</x:v>
+        <x:v>TEST-S03-005</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="35" t="str">
-        <x:v>S05-ACCESSORY-001</x:v>
+        <x:v>S03-REPAIR-001</x:v>
       </x:c>
       <x:c r="B49" s="36" t="str">
-        <x:v>S05</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C49" s="36" t="str">
-        <x:v>产品质量与型式资料</x:v>
+        <x:v>返修方案与记录</x:v>
       </x:c>
       <x:c r="D49" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1381,38 +1566,38 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F49" s="37" t="str">
-        <x:v>TEST-S05-002</x:v>
+        <x:v>TEST-S03-006</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="35" t="str">
-        <x:v>S05-INSTALL-001</x:v>
+        <x:v>S03-NDT-REPEAT-001</x:v>
       </x:c>
       <x:c r="B50" s="36" t="str">
-        <x:v>S05</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C50" s="36" t="str">
-        <x:v>安全附件到货安装记录</x:v>
+        <x:v>返修复检合格报告</x:v>
       </x:c>
       <x:c r="D50" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>DOCX</x:v>
       </x:c>
       <x:c r="E50" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F50" s="37" t="str">
-        <x:v>TEST-S05-003</x:v>
+        <x:v>TEST-S03-007</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="35" t="str">
-        <x:v>S05-PSV-001</x:v>
+        <x:v>S03-PWHT-001</x:v>
       </x:c>
       <x:c r="B51" s="36" t="str">
-        <x:v>S05</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C51" s="36" t="str">
-        <x:v>安全阀校验报告</x:v>
+        <x:v>热处理工艺与仪表</x:v>
       </x:c>
       <x:c r="D51" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1421,18 +1606,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F51" s="37" t="str">
-        <x:v>TEST-S05-004</x:v>
+        <x:v>TEST-S03-008</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="35" t="str">
-        <x:v>S05-ESDV-001</x:v>
+        <x:v>S03-PWHT-RECORD-001</x:v>
       </x:c>
       <x:c r="B52" s="36" t="str">
-        <x:v>S05</x:v>
+        <x:v>S03</x:v>
       </x:c>
       <x:c r="C52" s="36" t="str">
-        <x:v>紧急切断阀与爆破片记录</x:v>
+        <x:v>热处理曲线与硬度记录</x:v>
       </x:c>
       <x:c r="D52" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -1441,18 +1626,18 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F52" s="37" t="str">
-        <x:v>TEST-S05-005</x:v>
+        <x:v>TEST-S03-009</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="35" t="str">
-        <x:v>S06-ANALYSIS-001</x:v>
+        <x:v>S04-DESIGN-001</x:v>
       </x:c>
       <x:c r="B53" s="36" t="str">
-        <x:v>S06</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C53" s="36" t="str">
-        <x:v>耐压替代设计论证与应力分析</x:v>
+        <x:v>穿越与阴极保护设计变更</x:v>
       </x:c>
       <x:c r="D53" s="36" t="str">
         <x:v>DOCX</x:v>
@@ -1461,78 +1646,78 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F53" s="37" t="str">
-        <x:v>QX201903S-13-Y-TEST-S06-001</x:v>
+        <x:v>QX201903S-13-Y-TEST-S04-001</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="35" t="str">
-        <x:v>S06-APPROVAL-001</x:v>
+        <x:v>S04-DIAGRAM-001</x:v>
       </x:c>
       <x:c r="B54" s="36" t="str">
-        <x:v>S06</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C54" s="36" t="str">
-        <x:v>耐压替代申请审批</x:v>
+        <x:v>穿越结构与焊缝布置图</x:v>
       </x:c>
       <x:c r="D54" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>PDF</x:v>
       </x:c>
       <x:c r="E54" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F54" s="37" t="str">
-        <x:v>TEST-S06-002</x:v>
+        <x:v>TEST-S04-002</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="35" t="str">
-        <x:v>S06-ALTERNATIVE-001</x:v>
+        <x:v>S04-EQUIP-001</x:v>
       </x:c>
       <x:c r="B55" s="36" t="str">
-        <x:v>S06</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C55" s="36" t="str">
-        <x:v>替代检验试验方案</x:v>
+        <x:v>设备材料台账</x:v>
       </x:c>
       <x:c r="D55" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E55" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F55" s="37" t="str">
-        <x:v>TEST-S06-003</x:v>
+        <x:v>TEST-S04-003</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="35" t="str">
-        <x:v>S06-NDT-001</x:v>
+        <x:v>S04-INSTALL-001</x:v>
       </x:c>
       <x:c r="B56" s="36" t="str">
-        <x:v>S06</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C56" s="36" t="str">
-        <x:v>百分百RT-MT报告与底片</x:v>
+        <x:v>穿越施工与安装记录</x:v>
       </x:c>
       <x:c r="D56" s="36" t="str">
-        <x:v>DOCX</x:v>
+        <x:v>XLSX</x:v>
       </x:c>
       <x:c r="E56" s="36" t="str">
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F56" s="37" t="str">
-        <x:v>TEST-S06-004</x:v>
+        <x:v>TEST-S04-004</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="35" t="str">
-        <x:v>S06-FINAL-001</x:v>
+        <x:v>S04-CP-001</x:v>
       </x:c>
       <x:c r="B57" s="36" t="str">
-        <x:v>S06</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C57" s="36" t="str">
-        <x:v>替代试验泄漏最终确认</x:v>
+        <x:v>防腐阴保调试记录</x:v>
       </x:c>
       <x:c r="D57" s="36" t="str">
         <x:v>XLSX</x:v>
@@ -1541,117 +1726,513 @@
         <x:v>PDF</x:v>
       </x:c>
       <x:c r="F57" s="37" t="str">
-        <x:v>TEST-S06-005</x:v>
+        <x:v>TEST-S04-005</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="35" t="str">
-        <x:v>V00-NODE-MATRIX-001</x:v>
+        <x:v>S04-PHOTO-001</x:v>
       </x:c>
       <x:c r="B58" s="36" t="str">
-        <x:v>V00</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C58" s="36" t="str">
-        <x:v>R01-R69资料覆盖矩阵</x:v>
+        <x:v>施工照片</x:v>
       </x:c>
       <x:c r="D58" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E58" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F58" s="37" t="str">
-        <x:v>TEST-V00-001</x:v>
+        <x:v>TEST-S04-006</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="35" t="str">
-        <x:v>V00-REQ-MATRIX-001</x:v>
+        <x:v>S04-PHOTO-002</x:v>
       </x:c>
       <x:c r="B59" s="36" t="str">
-        <x:v>V00</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C59" s="36" t="str">
-        <x:v>166项资料要求覆盖明细</x:v>
+        <x:v>穿越开挖与就位核验图</x:v>
       </x:c>
       <x:c r="D59" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E59" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F59" s="37" t="str">
-        <x:v>TEST-V00-002</x:v>
+        <x:v>TEST-S04-007</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="35" t="str">
-        <x:v>V00-SOURCE-DIFF-001</x:v>
+        <x:v>S04-PHOTO-003</x:v>
       </x:c>
       <x:c r="B60" s="36" t="str">
-        <x:v>V00</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="C60" s="36" t="str">
-        <x:v>资料来源与差异台账</x:v>
+        <x:v>套管防腐绝缘核验图</x:v>
       </x:c>
       <x:c r="D60" s="36" t="str">
-        <x:v>XLSX</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="E60" s="36" t="str">
-        <x:v>PDF</x:v>
+        <x:v>JPG</x:v>
       </x:c>
       <x:c r="F60" s="37" t="str">
-        <x:v>TEST-V00-003</x:v>
+        <x:v>TEST-S04-008</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="35" t="str">
+        <x:v>S04-PHOTO-004</x:v>
+      </x:c>
+      <x:c r="B61" s="36" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="C61" s="36" t="str">
+        <x:v>绝缘支撑安装核验图</x:v>
+      </x:c>
+      <x:c r="D61" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="E61" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="F61" s="37" t="str">
+        <x:v>TEST-S04-009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="35" t="str">
+        <x:v>S04-PHOTO-005</x:v>
+      </x:c>
+      <x:c r="B62" s="36" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="C62" s="36" t="str">
+        <x:v>穿越焊接连接核验图</x:v>
+      </x:c>
+      <x:c r="D62" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="E62" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="F62" s="37" t="str">
+        <x:v>TEST-S04-010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="35" t="str">
+        <x:v>S04-PHOTO-006</x:v>
+      </x:c>
+      <x:c r="B63" s="36" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="C63" s="36" t="str">
+        <x:v>穿越布管完成核验图</x:v>
+      </x:c>
+      <x:c r="D63" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="E63" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="F63" s="37" t="str">
+        <x:v>TEST-S04-011</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="35" t="str">
+        <x:v>S05-DESIGN-001</x:v>
+      </x:c>
+      <x:c r="B64" s="36" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="C64" s="36" t="str">
+        <x:v>安全附件设计变更与选型</x:v>
+      </x:c>
+      <x:c r="D64" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E64" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F64" s="37" t="str">
+        <x:v>QX201903S-13-Y-TEST-S05-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="35" t="str">
+        <x:v>S05-ACCESSORY-001</x:v>
+      </x:c>
+      <x:c r="B65" s="36" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="C65" s="36" t="str">
+        <x:v>产品质量与型式资料</x:v>
+      </x:c>
+      <x:c r="D65" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E65" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F65" s="37" t="str">
+        <x:v>TEST-S05-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="35" t="str">
+        <x:v>S05-INSTALL-001</x:v>
+      </x:c>
+      <x:c r="B66" s="36" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="C66" s="36" t="str">
+        <x:v>安全附件到货安装记录</x:v>
+      </x:c>
+      <x:c r="D66" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E66" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F66" s="37" t="str">
+        <x:v>TEST-S05-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="35" t="str">
+        <x:v>S05-PSV-001</x:v>
+      </x:c>
+      <x:c r="B67" s="36" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="C67" s="36" t="str">
+        <x:v>安全阀校验报告</x:v>
+      </x:c>
+      <x:c r="D67" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E67" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F67" s="37" t="str">
+        <x:v>TEST-S05-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="35" t="str">
+        <x:v>S05-ESDV-001</x:v>
+      </x:c>
+      <x:c r="B68" s="36" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="C68" s="36" t="str">
+        <x:v>紧急切断阀与爆破片记录</x:v>
+      </x:c>
+      <x:c r="D68" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E68" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F68" s="37" t="str">
+        <x:v>TEST-S05-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="35" t="str">
+        <x:v>S06-ANALYSIS-001</x:v>
+      </x:c>
+      <x:c r="B69" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C69" s="36" t="str">
+        <x:v>耐压替代设计论证与应力分析</x:v>
+      </x:c>
+      <x:c r="D69" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E69" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F69" s="37" t="str">
+        <x:v>QX201903S-13-Y-TEST-S06-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
+      <x:c r="A70" s="35" t="str">
+        <x:v>S06-APPROVAL-001</x:v>
+      </x:c>
+      <x:c r="B70" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C70" s="36" t="str">
+        <x:v>耐压替代申请审批</x:v>
+      </x:c>
+      <x:c r="D70" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E70" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F70" s="37" t="str">
+        <x:v>TEST-S06-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="35" t="str">
+        <x:v>S06-ALTERNATIVE-001</x:v>
+      </x:c>
+      <x:c r="B71" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C71" s="36" t="str">
+        <x:v>替代检验试验方案</x:v>
+      </x:c>
+      <x:c r="D71" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E71" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F71" s="37" t="str">
+        <x:v>TEST-S06-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="35" t="str">
+        <x:v>S06-NDT-001</x:v>
+      </x:c>
+      <x:c r="B72" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C72" s="36" t="str">
+        <x:v>百分百RT-MT报告与底片</x:v>
+      </x:c>
+      <x:c r="D72" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E72" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F72" s="37" t="str">
+        <x:v>TEST-S06-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="35" t="str">
+        <x:v>S06-FINAL-001</x:v>
+      </x:c>
+      <x:c r="B73" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C73" s="36" t="str">
+        <x:v>替代试验泄漏最终确认</x:v>
+      </x:c>
+      <x:c r="D73" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E73" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F73" s="37" t="str">
+        <x:v>TEST-S06-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="35" t="str">
+        <x:v>S06-FILM-001</x:v>
+      </x:c>
+      <x:c r="B74" s="36" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="C74" s="36" t="str">
+        <x:v>最终封闭焊口射线检测模拟底片</x:v>
+      </x:c>
+      <x:c r="D74" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="E74" s="36" t="str">
+        <x:v>JPG</x:v>
+      </x:c>
+      <x:c r="F74" s="37" t="str">
+        <x:v>TEST-S06-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="35" t="str">
+        <x:v>V00-NODE-MATRIX-001</x:v>
+      </x:c>
+      <x:c r="B75" s="36" t="str">
+        <x:v>V00</x:v>
+      </x:c>
+      <x:c r="C75" s="36" t="str">
+        <x:v>R01-R69资料覆盖矩阵</x:v>
+      </x:c>
+      <x:c r="D75" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E75" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F75" s="37" t="str">
+        <x:v>TEST-V00-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="35" t="str">
+        <x:v>V00-REQ-MATRIX-001</x:v>
+      </x:c>
+      <x:c r="B76" s="36" t="str">
+        <x:v>V00</x:v>
+      </x:c>
+      <x:c r="C76" s="36" t="str">
+        <x:v>166项资料要求覆盖明细</x:v>
+      </x:c>
+      <x:c r="D76" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E76" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F76" s="37" t="str">
+        <x:v>TEST-V00-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="35" t="str">
+        <x:v>V00-SOURCE-DIFF-001</x:v>
+      </x:c>
+      <x:c r="B77" s="36" t="str">
+        <x:v>V00</x:v>
+      </x:c>
+      <x:c r="C77" s="36" t="str">
+        <x:v>资料来源与差异台账</x:v>
+      </x:c>
+      <x:c r="D77" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E77" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F77" s="37" t="str">
+        <x:v>TEST-V00-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="35" t="str">
         <x:v>V00-CHECKSUM-001</x:v>
       </x:c>
-      <x:c r="B61" s="36" t="str">
+      <x:c r="B78" s="36" t="str">
         <x:v>V00</x:v>
       </x:c>
-      <x:c r="C61" s="36" t="str">
+      <x:c r="C78" s="36" t="str">
         <x:v>文件校验清单</x:v>
       </x:c>
-      <x:c r="D61" s="36" t="str">
-        <x:v>XLSX</x:v>
-      </x:c>
-      <x:c r="E61" s="36" t="str">
-        <x:v>PDF</x:v>
-      </x:c>
-      <x:c r="F61" s="37" t="str">
+      <x:c r="D78" s="36" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E78" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F78" s="37" t="str">
         <x:v>TEST-V00-004</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="15" hidden="0" customHeight="1">
-      <x:c r="A62" s="38" t="str">
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="35" t="str">
         <x:v>V00-REPORT-001</x:v>
       </x:c>
-      <x:c r="B62" s="39" t="str">
+      <x:c r="B79" s="36" t="str">
         <x:v>V00</x:v>
       </x:c>
-      <x:c r="C62" s="39" t="str">
+      <x:c r="C79" s="36" t="str">
         <x:v>资料包完整性检查报告</x:v>
       </x:c>
-      <x:c r="D62" s="39" t="str">
-        <x:v>DOCX</x:v>
-      </x:c>
-      <x:c r="E62" s="39" t="str">
-        <x:v>PDF</x:v>
-      </x:c>
-      <x:c r="F62" s="40" t="str">
+      <x:c r="D79" s="36" t="str">
+        <x:v>DOCX</x:v>
+      </x:c>
+      <x:c r="E79" s="36" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F79" s="37" t="str">
         <x:v>TEST-V00-005</x:v>
       </x:c>
     </x:row>
-    <x:row r="63"/>
-    <x:row r="64"/>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="38" t="str">
+        <x:v>V00-R69-001</x:v>
+      </x:c>
+      <x:c r="B80" s="39" t="str">
+        <x:v>V00</x:v>
+      </x:c>
+      <x:c r="C80" s="39" t="str">
+        <x:v>R69质量保证体系实施状况工作流执行记录</x:v>
+      </x:c>
+      <x:c r="D80" s="39" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+      <x:c r="E80" s="39" t="str">
+        <x:v>PDF</x:v>
+      </x:c>
+      <x:c r="F80" s="40" t="str">
+        <x:v>TEST-V00-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81"/>
+    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="A82" s="60" t="str">
+        <x:v>电子签署（测试）｜资料验收测试专用章</x:v>
+      </x:c>
+      <x:c r="B82" s="61"/>
+      <x:c r="C82" s="61"/>
+      <x:c r="D82" s="61"/>
+      <x:c r="E82" s="61"/>
+      <x:c r="F82" s="62"/>
+    </x:row>
+    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="A83" s="63"/>
+      <x:c r="B83" s="64"/>
+      <x:c r="C83" s="64"/>
+      <x:c r="D83" s="64"/>
+      <x:c r="E83" s="64"/>
+      <x:c r="F83" s="65"/>
+    </x:row>
+    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="A84" s="63"/>
+      <x:c r="B84" s="64"/>
+      <x:c r="C84" s="64"/>
+      <x:c r="D84" s="64"/>
+      <x:c r="E84" s="64"/>
+      <x:c r="F84" s="65"/>
+    </x:row>
+    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="A85" s="66"/>
+      <x:c r="B85" s="67"/>
+      <x:c r="C85" s="67"/>
+      <x:c r="D85" s="67"/>
+      <x:c r="E85" s="67"/>
+      <x:c r="F85" s="68"/>
+    </x:row>
+    <x:row r="86"/>
+    <x:row r="87"/>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A82:C82"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="A5:F62">
+  <x:conditionalFormatting sqref="A5:F80">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>OR(ISNUMBER(SEARCH("不合格",A5)),ISNUMBER(SEARCH("异常",A5)))</x:formula>
     </x:cfRule>
@@ -1660,6 +2241,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12faa36e2ad1498a"/>
 </x:worksheet>
 </file>
 
@@ -1670,6 +2252,8 @@
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18" hidden="0" customHeight="1">
@@ -1678,6 +2262,8 @@
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
     </x:row>
     <x:row r="2" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1685,6 +2271,8 @@
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
+      <x:c r="D2" s="9"/>
+      <x:c r="E2" s="9"/>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1703,10 +2291,10 @@
         <x:v>逻辑资料</x:v>
       </x:c>
       <x:c r="B5" s="33" t="n">
-        <x:v>58</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>58，符合</x:v>
+        <x:v>76，符合</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1714,31 +2302,85 @@
         <x:v>物理文件</x:v>
       </x:c>
       <x:c r="B6" s="36" t="n">
-        <x:v>114</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C6" s="37" t="str">
-        <x:v>114，符合</x:v>
+        <x:v>136，符合</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="38" t="str">
+      <x:c r="A7" s="35" t="str">
+        <x:v>引用原始PDF</x:v>
+      </x:c>
+      <x:c r="B7" s="36" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C7" s="37" t="str">
+        <x:v>12，符合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>验收证据域文件</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="n">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="C8" s="37" t="str">
+        <x:v>148，符合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="38" t="str">
         <x:v>资料要求</x:v>
       </x:c>
-      <x:c r="B7" s="39" t="n">
+      <x:c r="B9" s="39" t="n">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="C7" s="40" t="str">
+      <x:c r="C9" s="40" t="str">
         <x:v>166，符合</x:v>
       </x:c>
     </x:row>
-    <x:row r="8"/>
-    <x:row r="9"/>
+    <x:row r="10"/>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="60" t="str">
+        <x:v>电子签署（测试）｜资料验收测试专用章</x:v>
+      </x:c>
+      <x:c r="B11" s="61"/>
+      <x:c r="C11" s="61"/>
+      <x:c r="D11" s="61"/>
+      <x:c r="E11" s="62"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="63"/>
+      <x:c r="B12" s="64"/>
+      <x:c r="C12" s="64"/>
+      <x:c r="D12" s="64"/>
+      <x:c r="E12" s="65"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="63"/>
+      <x:c r="B13" s="64"/>
+      <x:c r="C13" s="64"/>
+      <x:c r="D13" s="64"/>
+      <x:c r="E13" s="65"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="66"/>
+      <x:c r="B14" s="67"/>
+      <x:c r="C14" s="67"/>
+      <x:c r="D14" s="67"/>
+      <x:c r="E14" s="68"/>
+    </x:row>
+    <x:row r="15"/>
+    <x:row r="16"/>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:C1"/>
-    <x:mergeCell ref="A2:C2"/>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A11:C11"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="A5:C7">
+  <x:conditionalFormatting sqref="A5:C9">
     <x:cfRule type="expression" dxfId="2" priority="1">
       <x:formula>OR(ISNUMBER(SEARCH("不合格",A5)),ISNUMBER(SEARCH("异常",A5)))</x:formula>
     </x:cfRule>
@@ -1747,5 +2389,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2202f2bb91af48d2"/>
 </x:worksheet>
 </file>
</xml_diff>